<commit_message>
Update 實價登錄 data to 32 transactions (2026/07/25 query)
Replace data/guoyang_boyu_實價登錄.xlsx with the latest export (28 ->
32 records) and regenerate the report. New transactions land on A16
(4F/15F), B1 (9F), and B6 (18F). B6 now joins the 坪數-spread flag
list — its new 18F transaction records 29.51坪 vs. the existing
22.48坪, a 7.03坪 gap.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019qMmeph4mJXozC5k1Nyzof
</commit_message>
<xml_diff>
--- a/data/guoyang_boyu_實價登錄.xlsx
+++ b/data/guoyang_boyu_實價登錄.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="149">
-  <si>
-    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,110 年 7 月 至115 年 7 月 ,建案名稱：國揚鉑御　　　　　　資料來源：不動產交易實價查詢服務網　2026年07月12日 11:00:43</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="163">
+  <si>
+    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,114 年 7 月 至115 年 7 月 ,建案名稱：國揚鉑御　　　　　　資料來源：不動產交易實價查詢服務網　2026年07月25日 12:22:28</t>
   </si>
   <si>
     <t>建物坐落</t>
@@ -76,12 +76,126 @@
     <t>鼓山區龍中段194地號</t>
   </si>
   <si>
+    <t>A棟16號</t>
+  </si>
+  <si>
+    <t>國揚鉑御</t>
+  </si>
+  <si>
+    <t>115/06/09　</t>
+  </si>
+  <si>
+    <t>1306</t>
+  </si>
+  <si>
+    <t>63.87</t>
+  </si>
+  <si>
+    <t>20.45</t>
+  </si>
+  <si>
+    <t>58.08%</t>
+  </si>
+  <si>
+    <t>住宅大樓(11層含以上有電梯)</t>
+  </si>
+  <si>
+    <t>　4/20　</t>
+  </si>
+  <si>
+    <t>房地(土地+建物)</t>
+  </si>
+  <si>
+    <t>土:1 建:1車:0</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>住家用</t>
+  </si>
+  <si>
+    <t>鋼筋混凝土造</t>
+  </si>
+  <si>
+    <t>B棟6號</t>
+  </si>
+  <si>
+    <t>115/06/06　</t>
+  </si>
+  <si>
+    <t>1799</t>
+  </si>
+  <si>
+    <t>68.46</t>
+  </si>
+  <si>
+    <t>29.51</t>
+  </si>
+  <si>
+    <t>40.84%</t>
+  </si>
+  <si>
+    <t>　18/20　</t>
+  </si>
+  <si>
+    <t>房地(土地+建物)+車位</t>
+  </si>
+  <si>
+    <t>土:1 建:1車:1</t>
+  </si>
+  <si>
+    <t>260</t>
+  </si>
+  <si>
+    <t>115/06/03　</t>
+  </si>
+  <si>
+    <t>1669</t>
+  </si>
+  <si>
+    <t>69.39</t>
+  </si>
+  <si>
+    <t>27.48</t>
+  </si>
+  <si>
+    <t>43.21%</t>
+  </si>
+  <si>
+    <t>　15/20　</t>
+  </si>
+  <si>
+    <t>250</t>
+  </si>
+  <si>
+    <t>B棟1號</t>
+  </si>
+  <si>
+    <t>2760</t>
+  </si>
+  <si>
+    <t>64.56</t>
+  </si>
+  <si>
+    <t>45.45</t>
+  </si>
+  <si>
+    <t>46.21%</t>
+  </si>
+  <si>
+    <t>　9/20　</t>
+  </si>
+  <si>
+    <t>3房2廳2衛</t>
+  </si>
+  <si>
+    <t>280</t>
+  </si>
+  <si>
     <t>A棟10號</t>
   </si>
   <si>
-    <t>國揚鉑御</t>
-  </si>
-  <si>
     <t>115/05/30　</t>
   </si>
   <si>
@@ -97,30 +211,9 @@
     <t>40.97%</t>
   </si>
   <si>
-    <t>住宅大樓(11層含以上有電梯)</t>
-  </si>
-  <si>
     <t>　5/20　</t>
   </si>
   <si>
-    <t>房地(土地+建物)+車位</t>
-  </si>
-  <si>
-    <t>土:1 建:1車:1</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>260</t>
-  </si>
-  <si>
-    <t>住家用</t>
-  </si>
-  <si>
-    <t>鋼筋混凝土造</t>
-  </si>
-  <si>
     <t>A棟9號</t>
   </si>
   <si>
@@ -139,9 +232,6 @@
     <t>270</t>
   </si>
   <si>
-    <t>A棟16號</t>
-  </si>
-  <si>
     <t>115/05/29　</t>
   </si>
   <si>
@@ -151,12 +241,6 @@
     <t>67.78</t>
   </si>
   <si>
-    <t>27.48</t>
-  </si>
-  <si>
-    <t>43.21%</t>
-  </si>
-  <si>
     <t>　11/20　</t>
   </si>
   <si>
@@ -181,15 +265,6 @@
     <t>47.74%</t>
   </si>
   <si>
-    <t>　18/20　</t>
-  </si>
-  <si>
-    <t>3房2廳2衛</t>
-  </si>
-  <si>
-    <t>280</t>
-  </si>
-  <si>
     <t>A棟13號</t>
   </si>
   <si>
@@ -253,9 +328,6 @@
     <t>　3/20　</t>
   </si>
   <si>
-    <t>250</t>
-  </si>
-  <si>
     <t>3161</t>
   </si>
   <si>
@@ -289,18 +361,6 @@
     <t>67.39</t>
   </si>
   <si>
-    <t>20.45</t>
-  </si>
-  <si>
-    <t>58.08%</t>
-  </si>
-  <si>
-    <t>房地(土地+建物)</t>
-  </si>
-  <si>
-    <t>土:1 建:1車:0</t>
-  </si>
-  <si>
     <t>1719</t>
   </si>
   <si>
@@ -334,9 +394,6 @@
     <t>60.39</t>
   </si>
   <si>
-    <t>　4/20　</t>
-  </si>
-  <si>
     <t>2597</t>
   </si>
   <si>
@@ -388,21 +445,9 @@
     <t>1874</t>
   </si>
   <si>
-    <t>B棟1號</t>
-  </si>
-  <si>
     <t>2910</t>
   </si>
   <si>
-    <t>68.46</t>
-  </si>
-  <si>
-    <t>45.45</t>
-  </si>
-  <si>
-    <t>46.21%</t>
-  </si>
-  <si>
     <t>2780</t>
   </si>
   <si>
@@ -446,9 +491,6 @@
   </si>
   <si>
     <t>72.89</t>
-  </si>
-  <si>
-    <t>B棟6號</t>
   </si>
   <si>
     <t>1431</t>
@@ -852,7 +894,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:R34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50.63408000000001" customWidth="1"/>
@@ -993,13 +1035,13 @@
         <v>31</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q3" s="1" t="s">
         <v>31</v>
@@ -1013,13 +1055,13 @@
         <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>36</v>
@@ -1037,25 +1079,25 @@
         <v>27</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q4" s="1" t="s">
         <v>31</v>
@@ -1069,49 +1111,49 @@
         <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q5" s="1" t="s">
         <v>31</v>
@@ -1125,49 +1167,49 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q6" s="1" t="s">
         <v>31</v>
@@ -1181,49 +1223,49 @@
         <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q7" s="1" t="s">
         <v>31</v>
@@ -1237,49 +1279,49 @@
         <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="K8" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q8" s="1" t="s">
         <v>31</v>
@@ -1293,49 +1335,49 @@
         <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q9" s="1" t="s">
         <v>31</v>
@@ -1349,49 +1391,49 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>26</v>
+        <v>82</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q10" s="1" t="s">
         <v>31</v>
@@ -1405,49 +1447,49 @@
         <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="N11" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="O11" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q11" s="1" t="s">
         <v>31</v>
@@ -1461,49 +1503,49 @@
         <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>49</v>
+        <v>90</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>53</v>
+        <v>93</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>54</v>
+        <v>94</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q12" s="1" t="s">
         <v>31</v>
@@ -1517,49 +1559,49 @@
         <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>93</v>
+        <v>41</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>94</v>
+        <v>42</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q13" s="1" t="s">
         <v>31</v>
@@ -1573,49 +1615,49 @@
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>55</v>
+        <v>103</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M14" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q14" s="1" t="s">
         <v>31</v>
@@ -1629,49 +1671,49 @@
         <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>68</v>
+        <v>106</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>69</v>
+        <v>107</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q15" s="1" t="s">
         <v>31</v>
@@ -1685,49 +1727,49 @@
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>44</v>
+        <v>111</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>46</v>
+        <v>82</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q16" s="1" t="s">
         <v>31</v>
@@ -1741,31 +1783,31 @@
         <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>29</v>
@@ -1774,16 +1816,16 @@
         <v>30</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q17" s="1" t="s">
         <v>31</v>
@@ -1797,49 +1839,49 @@
         <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>74</v>
+        <v>40</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q18" s="1" t="s">
         <v>31</v>
@@ -1853,7 +1895,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>21</v>
@@ -1862,40 +1904,40 @@
         <v>109</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>74</v>
+        <v>119</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q19" s="1" t="s">
         <v>31</v>
@@ -1909,49 +1951,49 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>114</v>
+        <v>74</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>115</v>
+        <v>47</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>116</v>
+        <v>48</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>117</v>
+        <v>75</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q20" s="1" t="s">
         <v>31</v>
@@ -1965,49 +2007,49 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>68</v>
+        <v>93</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>120</v>
+        <v>28</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q21" s="1" t="s">
         <v>31</v>
@@ -2021,49 +2063,49 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>121</v>
+        <v>90</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>37</v>
+        <v>127</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>38</v>
+        <v>93</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q22" s="1" t="s">
         <v>31</v>
@@ -2077,49 +2119,49 @@
         <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>124</v>
+        <v>83</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>127</v>
+        <v>106</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>128</v>
+        <v>107</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>55</v>
+        <v>99</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q23" s="1" t="s">
         <v>31</v>
@@ -2133,49 +2175,49 @@
         <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>65</v>
+        <v>131</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>68</v>
+        <v>134</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>69</v>
+        <v>135</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q24" s="1" t="s">
         <v>31</v>
@@ -2189,49 +2231,49 @@
         <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>68</v>
+        <v>93</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>55</v>
+        <v>139</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q25" s="1" t="s">
         <v>31</v>
@@ -2245,49 +2287,49 @@
         <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>136</v>
+        <v>68</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>26</v>
+        <v>70</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>106</v>
+        <v>65</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M26" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q26" s="1" t="s">
         <v>31</v>
@@ -2301,49 +2343,49 @@
         <v>19</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>138</v>
+        <v>37</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>84</v>
+        <v>40</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q27" s="1" t="s">
         <v>31</v>
@@ -2357,49 +2399,49 @@
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>49</v>
+        <v>90</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>53</v>
+        <v>93</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>54</v>
+        <v>94</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q28" s="1" t="s">
         <v>31</v>
@@ -2413,49 +2455,49 @@
         <v>19</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q29" s="1" t="s">
         <v>31</v>
@@ -2469,54 +2511,278 @@
         <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>147</v>
+        <v>63</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>148</v>
+        <v>64</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="K30" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="M30" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N30" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="P30" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q30" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R30" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="G31" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="L30" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="M30" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N30" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="P30" s="1" t="s">
+      <c r="I31" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="N31" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="P31" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q31" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R31" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="P32" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q32" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R32" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N33" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="P33" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q33" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R33" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="Q30" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="R30" s="1" t="s">
+      <c r="C34" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L34" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M34" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N34" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="P34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q34" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R34" s="1" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 實價登錄 data to 34 transactions (2026/08/09 query)
Replace data/guoyang_boyu_實價登錄.xlsx with the latest export (32 ->
34 records) and regenerate. New transactions: A13 18F (3,319萬) and
B2 2F (1,380萬) — B2's first-ever sale, so it now shows a real
registry-based 坪數 instead of the spec-sheet estimate. Move
NEW_SINCE_DATE to 115/06/09 (the previous snapshot's newest date) so
just these two are highlighted this round.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019qMmeph4mJXozC5k1Nyzof
</commit_message>
<xml_diff>
--- a/data/guoyang_boyu_實價登錄.xlsx
+++ b/data/guoyang_boyu_實價登錄.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="163">
-  <si>
-    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,114 年 7 月 至115 年 7 月 ,建案名稱：國揚鉑御　　　　　　資料來源：不動產交易實價查詢服務網　2026年07月25日 12:22:28</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="171">
+  <si>
+    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,114 年 7 月 至115 年 7 月 ,建案名稱：國揚鉑御　　　　　　資料來源：不動產交易實價查詢服務網　2026年08月09日 14:48:42</t>
   </si>
   <si>
     <t>建物坐落</t>
@@ -76,12 +76,84 @@
     <t>鼓山區龍中段194地號</t>
   </si>
   <si>
+    <t>A棟13號</t>
+  </si>
+  <si>
+    <t>國揚鉑御</t>
+  </si>
+  <si>
+    <t>115/06/20　</t>
+  </si>
+  <si>
+    <t>3319</t>
+  </si>
+  <si>
+    <t>74.39</t>
+  </si>
+  <si>
+    <t>48.02</t>
+  </si>
+  <si>
+    <t>46.98%</t>
+  </si>
+  <si>
+    <t>住宅大樓(11層含以上有電梯)</t>
+  </si>
+  <si>
+    <t>　18/20　</t>
+  </si>
+  <si>
+    <t>房地(土地+建物)+車位</t>
+  </si>
+  <si>
+    <t>土:1 建:1車:1</t>
+  </si>
+  <si>
+    <t>3房2廳2衛</t>
+  </si>
+  <si>
+    <t>270</t>
+  </si>
+  <si>
+    <t>住家用</t>
+  </si>
+  <si>
+    <t>鋼筋混凝土造</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>B棟2號</t>
+  </si>
+  <si>
+    <t>115/06/19　</t>
+  </si>
+  <si>
+    <t>1380</t>
+  </si>
+  <si>
+    <t>61.38</t>
+  </si>
+  <si>
+    <t>22.48</t>
+  </si>
+  <si>
+    <t>53.62%</t>
+  </si>
+  <si>
+    <t>　2/20　</t>
+  </si>
+  <si>
+    <t>房地(土地+建物)</t>
+  </si>
+  <si>
+    <t>土:1 建:1車:0</t>
+  </si>
+  <si>
     <t>A棟16號</t>
   </si>
   <si>
-    <t>國揚鉑御</t>
-  </si>
-  <si>
     <t>115/06/09　</t>
   </si>
   <si>
@@ -97,27 +169,9 @@
     <t>58.08%</t>
   </si>
   <si>
-    <t>住宅大樓(11層含以上有電梯)</t>
-  </si>
-  <si>
     <t>　4/20　</t>
   </si>
   <si>
-    <t>房地(土地+建物)</t>
-  </si>
-  <si>
-    <t>土:1 建:1車:0</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>住家用</t>
-  </si>
-  <si>
-    <t>鋼筋混凝土造</t>
-  </si>
-  <si>
     <t>B棟6號</t>
   </si>
   <si>
@@ -136,15 +190,6 @@
     <t>40.84%</t>
   </si>
   <si>
-    <t>　18/20　</t>
-  </si>
-  <si>
-    <t>房地(土地+建物)+車位</t>
-  </si>
-  <si>
-    <t>土:1 建:1車:1</t>
-  </si>
-  <si>
     <t>260</t>
   </si>
   <si>
@@ -187,9 +232,6 @@
     <t>　9/20　</t>
   </si>
   <si>
-    <t>3房2廳2衛</t>
-  </si>
-  <si>
     <t>280</t>
   </si>
   <si>
@@ -229,9 +271,6 @@
     <t>40.63%</t>
   </si>
   <si>
-    <t>270</t>
-  </si>
-  <si>
     <t>115/05/29　</t>
   </si>
   <si>
@@ -265,9 +304,6 @@
     <t>47.74%</t>
   </si>
   <si>
-    <t>A棟13號</t>
-  </si>
-  <si>
     <t>115/05/23　</t>
   </si>
   <si>
@@ -334,12 +370,6 @@
     <t>70.29</t>
   </si>
   <si>
-    <t>48.02</t>
-  </si>
-  <si>
-    <t>46.98%</t>
-  </si>
-  <si>
     <t>　8/20　</t>
   </si>
   <si>
@@ -497,12 +527,6 @@
   </si>
   <si>
     <t>63.65</t>
-  </si>
-  <si>
-    <t>22.48</t>
-  </si>
-  <si>
-    <t>53.62%</t>
   </si>
 </sst>
 </file>
@@ -894,7 +918,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R34"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50.63408000000001" customWidth="1"/>
@@ -1035,19 +1059,19 @@
         <v>31</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -1055,55 +1079,55 @@
         <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -1111,55 +1135,55 @@
         <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="M5" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -1167,55 +1191,55 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>58</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
@@ -1223,55 +1247,55 @@
         <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="I7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N7" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="K7" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="O7" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
@@ -1285,7 +1309,7 @@
         <v>21</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>67</v>
@@ -1303,31 +1327,31 @@
         <v>27</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M8" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
@@ -1335,55 +1359,55 @@
         <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -1391,55 +1415,55 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="K10" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
@@ -1447,55 +1471,55 @@
         <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>83</v>
+        <v>45</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="H11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="I11" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J11" s="1" t="s">
+      <c r="K11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N11" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="K11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="O11" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
@@ -1509,49 +1533,49 @@
         <v>21</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
@@ -1559,7 +1583,7 @@
         <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>21</v>
@@ -1574,40 +1598,40 @@
         <v>98</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -1615,55 +1639,55 @@
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>59</v>
+        <v>102</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>63</v>
+        <v>105</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>64</v>
+        <v>106</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M14" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
@@ -1671,55 +1695,55 @@
         <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
@@ -1727,55 +1751,55 @@
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>81</v>
-      </c>
       <c r="H16" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
@@ -1789,13 +1813,13 @@
         <v>21</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>25</v>
@@ -1807,7 +1831,7 @@
         <v>27</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>29</v>
@@ -1819,19 +1843,19 @@
         <v>31</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
@@ -1839,55 +1863,55 @@
         <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>47</v>
+        <v>94</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>40</v>
+        <v>122</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M18" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
@@ -1895,55 +1919,55 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>93</v>
+        <v>49</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
@@ -1951,55 +1975,55 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>74</v>
+        <v>126</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
@@ -2007,55 +2031,55 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>28</v>
+        <v>129</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R21" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
@@ -2063,55 +2087,55 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>90</v>
+        <v>130</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>94</v>
+        <v>63</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
@@ -2119,55 +2143,55 @@
         <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="G23" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="H23" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="H23" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="I23" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>99</v>
+        <v>51</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q23" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R23" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
@@ -2175,55 +2199,55 @@
         <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>131</v>
+        <v>102</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>134</v>
+        <v>105</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>135</v>
+        <v>106</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>136</v>
+        <v>111</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q24" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R24" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
@@ -2231,55 +2255,55 @@
         <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q25" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
@@ -2287,55 +2311,55 @@
         <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>142</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>68</v>
+        <v>143</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>69</v>
+        <v>144</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>70</v>
+        <v>145</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>65</v>
+        <v>146</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M26" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
@@ -2343,55 +2367,55 @@
         <v>19</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>51</v>
+        <v>102</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>37</v>
+        <v>148</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>54</v>
+        <v>105</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>40</v>
+        <v>149</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N27" s="1" t="s">
         <v>58</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q27" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R27" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
@@ -2399,55 +2423,55 @@
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>90</v>
+        <v>150</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>145</v>
+        <v>82</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>146</v>
+        <v>79</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="N28" s="1" t="s">
         <v>58</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q28" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R28" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
@@ -2455,55 +2479,55 @@
         <v>19</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>148</v>
+        <v>55</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q29" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R29" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
@@ -2511,55 +2535,55 @@
         <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>140</v>
+        <v>102</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>63</v>
+        <v>105</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>64</v>
+        <v>106</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>28</v>
+        <v>156</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M30" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O30" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q30" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R30" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
@@ -2567,55 +2591,55 @@
         <v>19</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>108</v>
+        <v>28</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q31" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R31" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
@@ -2623,55 +2647,55 @@
         <v>19</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="G32" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>81</v>
-      </c>
       <c r="H32" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>108</v>
+        <v>51</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q32" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R32" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
@@ -2679,55 +2703,55 @@
         <v>19</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>63</v>
+        <v>105</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>64</v>
+        <v>106</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="M33" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R33" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
@@ -2735,31 +2759,31 @@
         <v>19</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>161</v>
+        <v>94</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>162</v>
+        <v>95</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="K34" s="1" t="s">
         <v>29</v>
@@ -2771,19 +2795,131 @@
         <v>31</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="O34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P34" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q34" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R34" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N35" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="P34" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q34" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="R34" s="1" t="s">
-        <v>31</v>
+      <c r="O35" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P35" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q35" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R35" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P36" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q36" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R36" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update 實價登錄 data to 37 transactions (2026/08/16 query)
Replace data/guoyang_boyu_實價登錄.xlsx with the latest export (34 ->
37 records) and regenerate. New transactions: A8 10F (3,358萬), A15
4F (1,546萬), B8 16F (2,685萬) — B8's first-ever sale, so it now shows
a real registry-based 坪數 instead of the spec-sheet estimate. Move
NEW_SINCE_DATE to 115/06/20 (the previous snapshot's newest date) so
just these three are highlighted this round.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019qMmeph4mJXozC5k1Nyzof
</commit_message>
<xml_diff>
--- a/data/guoyang_boyu_實價登錄.xlsx
+++ b/data/guoyang_boyu_實價登錄.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="171">
-  <si>
-    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,114 年 7 月 至115 年 7 月 ,建案名稱：國揚鉑御　　　　　　資料來源：不動產交易實價查詢服務網　2026年08月09日 14:48:42</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="181">
+  <si>
+    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,110 年 7 月 至115 年 8 月 ,建案名稱：國揚　　　　　　資料來源：不動產交易實價查詢服務網　2026年08月16日 16:32:42</t>
   </si>
   <si>
     <t>建物坐落</t>
@@ -76,12 +76,102 @@
     <t>鼓山區龍中段194地號</t>
   </si>
   <si>
+    <t>B棟8號</t>
+  </si>
+  <si>
+    <t>國揚鉑御</t>
+  </si>
+  <si>
+    <t>115/06/28　</t>
+  </si>
+  <si>
+    <t>2685</t>
+  </si>
+  <si>
+    <t>64.58</t>
+  </si>
+  <si>
+    <t>44.43</t>
+  </si>
+  <si>
+    <t>45.70%</t>
+  </si>
+  <si>
+    <t>住宅大樓(11層含以上有電梯)</t>
+  </si>
+  <si>
+    <t>　16/20　</t>
+  </si>
+  <si>
+    <t>房地(土地+建物)+車位</t>
+  </si>
+  <si>
+    <t>土:1 建:1車:1</t>
+  </si>
+  <si>
+    <t>3房2廳2衛</t>
+  </si>
+  <si>
+    <t>270</t>
+  </si>
+  <si>
+    <t>住家用</t>
+  </si>
+  <si>
+    <t>鋼筋混凝土造</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>A棟15號</t>
+  </si>
+  <si>
+    <t>1546</t>
+  </si>
+  <si>
+    <t>63.87</t>
+  </si>
+  <si>
+    <t>27.48</t>
+  </si>
+  <si>
+    <t>43.21%</t>
+  </si>
+  <si>
+    <t>　4/20　</t>
+  </si>
+  <si>
+    <t>240</t>
+  </si>
+  <si>
+    <t>A棟8號</t>
+  </si>
+  <si>
+    <t>115/06/23　</t>
+  </si>
+  <si>
+    <t>3358</t>
+  </si>
+  <si>
+    <t>69.37</t>
+  </si>
+  <si>
+    <t>51.41</t>
+  </si>
+  <si>
+    <t>47.74%</t>
+  </si>
+  <si>
+    <t>　10/20　</t>
+  </si>
+  <si>
+    <t>280</t>
+  </si>
+  <si>
     <t>A棟13號</t>
   </si>
   <si>
-    <t>國揚鉑御</t>
-  </si>
-  <si>
     <t>115/06/20　</t>
   </si>
   <si>
@@ -97,33 +187,9 @@
     <t>46.98%</t>
   </si>
   <si>
-    <t>住宅大樓(11層含以上有電梯)</t>
-  </si>
-  <si>
     <t>　18/20　</t>
   </si>
   <si>
-    <t>房地(土地+建物)+車位</t>
-  </si>
-  <si>
-    <t>土:1 建:1車:1</t>
-  </si>
-  <si>
-    <t>3房2廳2衛</t>
-  </si>
-  <si>
-    <t>270</t>
-  </si>
-  <si>
-    <t>住家用</t>
-  </si>
-  <si>
-    <t>鋼筋混凝土造</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>B棟2號</t>
   </si>
   <si>
@@ -160,18 +226,12 @@
     <t>1306</t>
   </si>
   <si>
-    <t>63.87</t>
-  </si>
-  <si>
     <t>20.45</t>
   </si>
   <si>
     <t>58.08%</t>
   </si>
   <si>
-    <t>　4/20　</t>
-  </si>
-  <si>
     <t>B棟6號</t>
   </si>
   <si>
@@ -202,12 +262,6 @@
     <t>69.39</t>
   </si>
   <si>
-    <t>27.48</t>
-  </si>
-  <si>
-    <t>43.21%</t>
-  </si>
-  <si>
     <t>　15/20　</t>
   </si>
   <si>
@@ -232,9 +286,6 @@
     <t>　9/20　</t>
   </si>
   <si>
-    <t>280</t>
-  </si>
-  <si>
     <t>A棟10號</t>
   </si>
   <si>
@@ -283,12 +334,6 @@
     <t>　11/20　</t>
   </si>
   <si>
-    <t>240</t>
-  </si>
-  <si>
-    <t>A棟8號</t>
-  </si>
-  <si>
     <t>115/05/24　</t>
   </si>
   <si>
@@ -298,12 +343,6 @@
     <t>72.88</t>
   </si>
   <si>
-    <t>51.41</t>
-  </si>
-  <si>
-    <t>47.74%</t>
-  </si>
-  <si>
     <t>115/05/23　</t>
   </si>
   <si>
@@ -337,9 +376,6 @@
     <t>45.51%</t>
   </si>
   <si>
-    <t>　10/20　</t>
-  </si>
-  <si>
     <t>115/05/22　</t>
   </si>
   <si>
@@ -406,9 +442,6 @@
     <t>　7/20　</t>
   </si>
   <si>
-    <t>A棟15號</t>
-  </si>
-  <si>
     <t>115/05/19　</t>
   </si>
   <si>
@@ -461,9 +494,6 @@
   </si>
   <si>
     <t>66.08</t>
-  </si>
-  <si>
-    <t>　16/20　</t>
   </si>
   <si>
     <t>A棟12號</t>
@@ -918,7 +948,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R36"/>
+  <dimension ref="A1:R39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50.63408000000001" customWidth="1"/>
@@ -1085,37 +1115,37 @@
         <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N4" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="O4" s="1" t="s">
         <v>33</v>
@@ -1135,43 +1165,43 @@
         <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="I5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="K5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N5" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>33</v>
@@ -1191,32 +1221,32 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="I6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="K6" s="1" t="s">
         <v>29</v>
       </c>
@@ -1224,10 +1254,10 @@
         <v>30</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>33</v>
@@ -1247,7 +1277,7 @@
         <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>21</v>
@@ -1274,16 +1304,16 @@
         <v>64</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="M7" s="1" t="s">
         <v>35</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>33</v>
@@ -1303,43 +1333,43 @@
         <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L8" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="M8" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>33</v>
@@ -1359,43 +1389,43 @@
         <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N9" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>33</v>
@@ -1415,43 +1445,43 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="K10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N10" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N10" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>33</v>
@@ -1471,31 +1501,31 @@
         <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="H11" s="1" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>29</v>
@@ -1504,10 +1534,10 @@
         <v>30</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>89</v>
+        <v>50</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>33</v>
@@ -1551,7 +1581,7 @@
         <v>27</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>28</v>
+        <v>96</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>29</v>
@@ -1560,10 +1590,10 @@
         <v>30</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>33</v>
@@ -1583,32 +1613,32 @@
         <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J13" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>101</v>
-      </c>
       <c r="K13" s="1" t="s">
         <v>29</v>
       </c>
@@ -1616,10 +1646,10 @@
         <v>30</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="O13" s="1" t="s">
         <v>33</v>
@@ -1639,13 +1669,13 @@
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>103</v>
@@ -1654,17 +1684,17 @@
         <v>104</v>
       </c>
       <c r="G14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J14" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="K14" s="1" t="s">
         <v>29</v>
       </c>
@@ -1672,10 +1702,10 @@
         <v>30</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>33</v>
@@ -1695,31 +1725,31 @@
         <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>90</v>
+        <v>43</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>110</v>
-      </c>
       <c r="G15" s="1" t="s">
-        <v>94</v>
+        <v>47</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>95</v>
+        <v>48</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>111</v>
+        <v>57</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>29</v>
@@ -1731,7 +1761,7 @@
         <v>31</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>33</v>
@@ -1751,32 +1781,32 @@
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="I16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J16" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="K16" s="1" t="s">
         <v>29</v>
       </c>
@@ -1784,10 +1814,10 @@
         <v>30</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="O16" s="1" t="s">
         <v>33</v>
@@ -1807,13 +1837,13 @@
         <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>20</v>
+        <v>115</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>116</v>
@@ -1822,16 +1852,16 @@
         <v>117</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>25</v>
+        <v>118</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>26</v>
+        <v>119</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>118</v>
+        <v>49</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>29</v>
@@ -1843,7 +1873,7 @@
         <v>31</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="O17" s="1" t="s">
         <v>33</v>
@@ -1863,31 +1893,31 @@
         <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>90</v>
+        <v>43</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>94</v>
+        <v>47</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>95</v>
+        <v>48</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K18" s="1" t="s">
         <v>29</v>
@@ -1899,7 +1929,7 @@
         <v>31</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="O18" s="1" t="s">
         <v>33</v>
@@ -1919,43 +1949,43 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>49</v>
+        <v>94</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>50</v>
+        <v>95</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="M19" s="1" t="s">
         <v>35</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>35</v>
+        <v>83</v>
       </c>
       <c r="O19" s="1" t="s">
         <v>33</v>
@@ -1975,31 +2005,31 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>28</v>
+        <v>130</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>29</v>
@@ -2008,10 +2038,10 @@
         <v>30</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>33</v>
@@ -2031,31 +2061,31 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>102</v>
+        <v>43</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>105</v>
+        <v>47</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>106</v>
+        <v>48</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>29</v>
@@ -2067,7 +2097,7 @@
         <v>31</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>33</v>
@@ -2087,7 +2117,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>130</v>
+        <v>67</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>21</v>
@@ -2096,34 +2126,34 @@
         <v>131</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>87</v>
+        <v>136</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>88</v>
+        <v>49</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="M22" s="1" t="s">
         <v>35</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="O22" s="1" t="s">
         <v>33</v>
@@ -2143,31 +2173,31 @@
         <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>102</v>
+        <v>67</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>105</v>
+        <v>39</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>106</v>
+        <v>40</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>29</v>
@@ -2176,10 +2206,10 @@
         <v>30</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="O23" s="1" t="s">
         <v>33</v>
@@ -2199,31 +2229,31 @@
         <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
       <c r="K24" s="1" t="s">
         <v>29</v>
@@ -2235,7 +2265,7 @@
         <v>31</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="O24" s="1" t="s">
         <v>33</v>
@@ -2255,31 +2285,31 @@
         <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>140</v>
+        <v>104</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="K25" s="1" t="s">
         <v>29</v>
@@ -2288,10 +2318,10 @@
         <v>30</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="O25" s="1" t="s">
         <v>33</v>
@@ -2311,31 +2341,31 @@
         <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>141</v>
+        <v>115</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>144</v>
+        <v>118</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>145</v>
+        <v>119</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>146</v>
+        <v>41</v>
       </c>
       <c r="K26" s="1" t="s">
         <v>29</v>
@@ -2347,7 +2377,7 @@
         <v>31</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="O26" s="1" t="s">
         <v>33</v>
@@ -2367,13 +2397,13 @@
         <v>19</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>147</v>
@@ -2382,16 +2412,16 @@
         <v>148</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>149</v>
+        <v>123</v>
       </c>
       <c r="K27" s="1" t="s">
         <v>29</v>
@@ -2403,7 +2433,7 @@
         <v>31</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="O27" s="1" t="s">
         <v>33</v>
@@ -2423,31 +2453,31 @@
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D28" s="1" t="s">
+      <c r="F28" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="G28" s="1" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>79</v>
+        <v>123</v>
       </c>
       <c r="K28" s="1" t="s">
         <v>29</v>
@@ -2456,10 +2486,10 @@
         <v>30</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="O28" s="1" t="s">
         <v>33</v>
@@ -2479,31 +2509,31 @@
         <v>19</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>66</v>
+        <v>152</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>153</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>55</v>
+        <v>154</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>69</v>
+        <v>155</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>70</v>
+        <v>156</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>28</v>
+        <v>157</v>
       </c>
       <c r="K29" s="1" t="s">
         <v>29</v>
@@ -2515,7 +2545,7 @@
         <v>31</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="O29" s="1" t="s">
         <v>33</v>
@@ -2535,31 +2565,31 @@
         <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>156</v>
+        <v>28</v>
       </c>
       <c r="K30" s="1" t="s">
         <v>29</v>
@@ -2571,7 +2601,7 @@
         <v>31</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="O30" s="1" t="s">
         <v>33</v>
@@ -2591,31 +2621,31 @@
         <v>19</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>102</v>
+        <v>160</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>158</v>
+        <v>99</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>28</v>
+        <v>96</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>29</v>
@@ -2624,10 +2654,10 @@
         <v>30</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>33</v>
@@ -2647,31 +2677,31 @@
         <v>19</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>150</v>
+        <v>84</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>161</v>
+        <v>75</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="K32" s="1" t="s">
         <v>29</v>
@@ -2680,10 +2710,10 @@
         <v>30</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="O32" s="1" t="s">
         <v>33</v>
@@ -2703,31 +2733,31 @@
         <v>19</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>118</v>
+        <v>166</v>
       </c>
       <c r="K33" s="1" t="s">
         <v>29</v>
@@ -2739,7 +2769,7 @@
         <v>31</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>33</v>
@@ -2759,31 +2789,31 @@
         <v>19</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>118</v>
+        <v>57</v>
       </c>
       <c r="K34" s="1" t="s">
         <v>29</v>
@@ -2795,7 +2825,7 @@
         <v>31</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="O34" s="1" t="s">
         <v>33</v>
@@ -2815,31 +2845,31 @@
         <v>19</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>107</v>
+        <v>41</v>
       </c>
       <c r="K35" s="1" t="s">
         <v>29</v>
@@ -2871,54 +2901,222 @@
         <v>19</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>52</v>
+        <v>115</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>40</v>
+        <v>118</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>41</v>
+        <v>119</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="K36" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P36" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q36" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R36" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L36" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="M36" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="O36" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="P36" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q36" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="R36" s="1" t="s">
+      <c r="C37" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N37" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P37" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q37" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R37" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L38" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M38" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N38" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P38" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q38" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R38" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L39" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M39" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N39" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O39" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P39" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q39" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R39" s="1" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 實價登錄 data to 41 transactions (2026/08/22 query)
Replace data/guoyang_boyu_實價登錄.xlsx with the latest export (37 ->
41 records) and regenerate. New transactions: A7 12F (3,171萬), A15
12F (1,396萬), A9 6F (1,854萬), B9 3F (2,528萬) — A7's first-ever sale,
so it now shows a real registry-based 坪數 (43.05坪) instead of the
spec-sheet estimate (41.00坪). Move NEW_SINCE_DATE to 115/06/28 (the
previous snapshot's newest date) so just these four are highlighted
this round.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019qMmeph4mJXozC5k1Nyzof
</commit_message>
<xml_diff>
--- a/data/guoyang_boyu_實價登錄.xlsx
+++ b/data/guoyang_boyu_實價登錄.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="181">
-  <si>
-    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,110 年 7 月 至115 年 8 月 ,建案名稱：國揚　　　　　　資料來源：不動產交易實價查詢服務網　2026年08月16日 16:32:42</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="195">
+  <si>
+    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,114 年 8 月 至115 年 8 月 ,建案名稱：國揚鉑御　　　　　　資料來源：不動產交易實價查詢服務網　2026年08月22日 13:59:31</t>
   </si>
   <si>
     <t>建物坐落</t>
@@ -76,12 +76,126 @@
     <t>鼓山區龍中段194地號</t>
   </si>
   <si>
+    <t>A棟9號</t>
+  </si>
+  <si>
+    <t>國揚鉑御</t>
+  </si>
+  <si>
+    <t>115/07/10　</t>
+  </si>
+  <si>
+    <t>1854</t>
+  </si>
+  <si>
+    <t>71.68</t>
+  </si>
+  <si>
+    <t>29.41</t>
+  </si>
+  <si>
+    <t>40.97%</t>
+  </si>
+  <si>
+    <t>住宅大樓(11層含以上有電梯)</t>
+  </si>
+  <si>
+    <t>　6/20　</t>
+  </si>
+  <si>
+    <t>房地(土地+建物)+車位</t>
+  </si>
+  <si>
+    <t>土:1 建:1車:1</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>250</t>
+  </si>
+  <si>
+    <t>住家用</t>
+  </si>
+  <si>
+    <t>鋼筋混凝土造</t>
+  </si>
+  <si>
+    <t>B棟9號</t>
+  </si>
+  <si>
+    <t>115/07/04　</t>
+  </si>
+  <si>
+    <t>2528</t>
+  </si>
+  <si>
+    <t>61.38</t>
+  </si>
+  <si>
+    <t>44.47</t>
+  </si>
+  <si>
+    <t>45.51%</t>
+  </si>
+  <si>
+    <t>　3/20　</t>
+  </si>
+  <si>
+    <t>3房2廳2衛</t>
+  </si>
+  <si>
+    <t>230</t>
+  </si>
+  <si>
+    <t>A棟15號</t>
+  </si>
+  <si>
+    <t>1396</t>
+  </si>
+  <si>
+    <t>68.27</t>
+  </si>
+  <si>
+    <t>20.45</t>
+  </si>
+  <si>
+    <t>58.08%</t>
+  </si>
+  <si>
+    <t>　12/20　</t>
+  </si>
+  <si>
+    <t>房地(土地+建物)</t>
+  </si>
+  <si>
+    <t>土:1 建:1車:0</t>
+  </si>
+  <si>
+    <t>A棟7號</t>
+  </si>
+  <si>
+    <t>115/07/01　</t>
+  </si>
+  <si>
+    <t>3171</t>
+  </si>
+  <si>
+    <t>67.17</t>
+  </si>
+  <si>
+    <t>50.08</t>
+  </si>
+  <si>
+    <t>47.58%</t>
+  </si>
+  <si>
+    <t>280</t>
+  </si>
+  <si>
     <t>B棟8號</t>
   </si>
   <si>
-    <t>國揚鉑御</t>
-  </si>
-  <si>
     <t>115/06/28　</t>
   </si>
   <si>
@@ -97,36 +211,12 @@
     <t>45.70%</t>
   </si>
   <si>
-    <t>住宅大樓(11層含以上有電梯)</t>
-  </si>
-  <si>
     <t>　16/20　</t>
   </si>
   <si>
-    <t>房地(土地+建物)+車位</t>
-  </si>
-  <si>
-    <t>土:1 建:1車:1</t>
-  </si>
-  <si>
-    <t>3房2廳2衛</t>
-  </si>
-  <si>
     <t>270</t>
   </si>
   <si>
-    <t>住家用</t>
-  </si>
-  <si>
-    <t>鋼筋混凝土造</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>A棟15號</t>
-  </si>
-  <si>
     <t>1546</t>
   </si>
   <si>
@@ -166,9 +256,6 @@
     <t>　10/20　</t>
   </si>
   <si>
-    <t>280</t>
-  </si>
-  <si>
     <t>A棟13號</t>
   </si>
   <si>
@@ -199,9 +286,6 @@
     <t>1380</t>
   </si>
   <si>
-    <t>61.38</t>
-  </si>
-  <si>
     <t>22.48</t>
   </si>
   <si>
@@ -211,12 +295,6 @@
     <t>　2/20　</t>
   </si>
   <si>
-    <t>房地(土地+建物)</t>
-  </si>
-  <si>
-    <t>土:1 建:1車:0</t>
-  </si>
-  <si>
     <t>A棟16號</t>
   </si>
   <si>
@@ -226,12 +304,6 @@
     <t>1306</t>
   </si>
   <si>
-    <t>20.45</t>
-  </si>
-  <si>
-    <t>58.08%</t>
-  </si>
-  <si>
     <t>B棟6號</t>
   </si>
   <si>
@@ -265,9 +337,6 @@
     <t>　15/20　</t>
   </si>
   <si>
-    <t>250</t>
-  </si>
-  <si>
     <t>B棟1號</t>
   </si>
   <si>
@@ -298,18 +367,9 @@
     <t>71.37</t>
   </si>
   <si>
-    <t>29.41</t>
-  </si>
-  <si>
-    <t>40.97%</t>
-  </si>
-  <si>
     <t>　5/20　</t>
   </si>
   <si>
-    <t>A棟9號</t>
-  </si>
-  <si>
     <t>1884</t>
   </si>
   <si>
@@ -361,21 +421,12 @@
     <t>　20/20　</t>
   </si>
   <si>
-    <t>B棟9號</t>
-  </si>
-  <si>
     <t>2672</t>
   </si>
   <si>
     <t>63.89</t>
   </si>
   <si>
-    <t>44.47</t>
-  </si>
-  <si>
-    <t>45.51%</t>
-  </si>
-  <si>
     <t>115/05/22　</t>
   </si>
   <si>
@@ -385,9 +436,6 @@
     <t>68.17</t>
   </si>
   <si>
-    <t>　6/20　</t>
-  </si>
-  <si>
     <t>115/05/21　</t>
   </si>
   <si>
@@ -397,9 +445,6 @@
     <t>70.39</t>
   </si>
   <si>
-    <t>　3/20　</t>
-  </si>
-  <si>
     <t>3161</t>
   </si>
   <si>
@@ -416,9 +461,6 @@
   </si>
   <si>
     <t>70.18</t>
-  </si>
-  <si>
-    <t>　12/20　</t>
   </si>
   <si>
     <t>1378</t>
@@ -948,7 +990,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R39"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50.63408000000001" customWidth="1"/>
@@ -1098,10 +1140,10 @@
         <v>34</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -1109,13 +1151,13 @@
         <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>37</v>
@@ -1142,10 +1184,10 @@
         <v>30</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O4" s="1" t="s">
         <v>33</v>
@@ -1154,10 +1196,10 @@
         <v>34</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -1165,13 +1207,13 @@
         <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>45</v>
@@ -1192,16 +1234,16 @@
         <v>49</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>33</v>
@@ -1210,10 +1252,10 @@
         <v>34</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -1221,31 +1263,31 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>29</v>
@@ -1254,10 +1296,10 @@
         <v>30</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>33</v>
@@ -1266,10 +1308,10 @@
         <v>34</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
@@ -1277,44 +1319,44 @@
         <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>65</v>
+        <v>29</v>
       </c>
       <c r="L7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="N7" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="M7" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="O7" s="1" t="s">
         <v>33</v>
       </c>
@@ -1322,10 +1364,10 @@
         <v>34</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
@@ -1333,43 +1375,43 @@
         <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="I8" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="K8" s="1" t="s">
-        <v>65</v>
+        <v>29</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>33</v>
@@ -1378,10 +1420,10 @@
         <v>34</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
@@ -1389,31 +1431,31 @@
         <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>29</v>
@@ -1422,10 +1464,10 @@
         <v>30</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>33</v>
@@ -1434,10 +1476,10 @@
         <v>34</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -1445,31 +1487,31 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>29</v>
@@ -1478,10 +1520,10 @@
         <v>30</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>33</v>
@@ -1490,10 +1532,10 @@
         <v>34</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
@@ -1501,43 +1543,43 @@
         <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="M11" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>33</v>
@@ -1546,10 +1588,10 @@
         <v>34</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
@@ -1557,43 +1599,43 @@
         <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>93</v>
+        <v>68</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>94</v>
+        <v>47</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>95</v>
+        <v>48</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>33</v>
@@ -1602,10 +1644,10 @@
         <v>34</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
@@ -1613,13 +1655,13 @@
         <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>98</v>
@@ -1637,7 +1679,7 @@
         <v>27</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>29</v>
@@ -1646,10 +1688,10 @@
         <v>30</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>32</v>
+        <v>102</v>
       </c>
       <c r="O13" s="1" t="s">
         <v>33</v>
@@ -1658,10 +1700,10 @@
         <v>34</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -1669,31 +1711,31 @@
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K14" s="1" t="s">
         <v>29</v>
@@ -1702,10 +1744,10 @@
         <v>30</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>33</v>
@@ -1714,10 +1756,10 @@
         <v>34</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
@@ -1725,31 +1767,31 @@
         <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>43</v>
+        <v>107</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>47</v>
+        <v>110</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>48</v>
+        <v>111</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>57</v>
+        <v>112</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>29</v>
@@ -1758,10 +1800,10 @@
         <v>30</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>33</v>
@@ -1770,10 +1812,10 @@
         <v>34</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
@@ -1781,31 +1823,31 @@
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>112</v>
+        <v>25</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>113</v>
+        <v>26</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>29</v>
@@ -1817,7 +1859,7 @@
         <v>31</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>50</v>
+        <v>102</v>
       </c>
       <c r="O16" s="1" t="s">
         <v>33</v>
@@ -1826,10 +1868,10 @@
         <v>34</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
@@ -1837,32 +1879,32 @@
         <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>115</v>
+        <v>20</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F17" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="K17" s="1" t="s">
         <v>29</v>
       </c>
@@ -1873,7 +1915,7 @@
         <v>31</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="O17" s="1" t="s">
         <v>33</v>
@@ -1882,10 +1924,10 @@
         <v>34</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
@@ -1893,31 +1935,31 @@
         <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="K18" s="1" t="s">
         <v>29</v>
@@ -1929,7 +1971,7 @@
         <v>31</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="O18" s="1" t="s">
         <v>33</v>
@@ -1938,10 +1980,10 @@
         <v>34</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
@@ -1949,31 +1991,31 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>127</v>
+        <v>86</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>29</v>
@@ -1982,10 +2024,10 @@
         <v>30</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="O19" s="1" t="s">
         <v>33</v>
@@ -1994,10 +2036,10 @@
         <v>34</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
@@ -2005,31 +2047,31 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>51</v>
+        <v>80</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>55</v>
+        <v>132</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>56</v>
+        <v>133</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>29</v>
@@ -2038,10 +2080,10 @@
         <v>30</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>33</v>
@@ -2050,10 +2092,10 @@
         <v>34</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
@@ -2061,31 +2103,31 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>134</v>
+        <v>79</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>29</v>
@@ -2094,10 +2136,10 @@
         <v>30</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>33</v>
@@ -2106,10 +2148,10 @@
         <v>34</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R21" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
@@ -2117,44 +2159,44 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>65</v>
+        <v>29</v>
       </c>
       <c r="L22" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="N22" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="M22" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N22" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="O22" s="1" t="s">
         <v>33</v>
       </c>
@@ -2162,10 +2204,10 @@
         <v>34</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
@@ -2173,31 +2215,31 @@
         <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>67</v>
+        <v>113</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>29</v>
@@ -2206,7 +2248,7 @@
         <v>30</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N23" s="1" t="s">
         <v>32</v>
@@ -2218,10 +2260,10 @@
         <v>34</v>
       </c>
       <c r="Q23" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R23" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
@@ -2229,31 +2271,31 @@
         <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>118</v>
+        <v>84</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>119</v>
+        <v>85</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="K24" s="1" t="s">
         <v>29</v>
@@ -2262,10 +2304,10 @@
         <v>30</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="O24" s="1" t="s">
         <v>33</v>
@@ -2274,10 +2316,10 @@
         <v>34</v>
       </c>
       <c r="Q24" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R24" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
@@ -2285,31 +2327,31 @@
         <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>104</v>
+        <v>148</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>105</v>
+        <v>49</v>
       </c>
       <c r="K25" s="1" t="s">
         <v>29</v>
@@ -2318,10 +2360,10 @@
         <v>30</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="O25" s="1" t="s">
         <v>33</v>
@@ -2330,10 +2372,10 @@
         <v>34</v>
       </c>
       <c r="Q25" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
@@ -2341,43 +2383,43 @@
         <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>115</v>
+        <v>93</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>118</v>
+        <v>47</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>119</v>
+        <v>48</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="M26" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>83</v>
+        <v>31</v>
       </c>
       <c r="O26" s="1" t="s">
         <v>33</v>
@@ -2386,10 +2428,10 @@
         <v>34</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
@@ -2397,31 +2439,31 @@
         <v>19</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>115</v>
+        <v>93</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>118</v>
+        <v>69</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>119</v>
+        <v>70</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>123</v>
+        <v>86</v>
       </c>
       <c r="K27" s="1" t="s">
         <v>29</v>
@@ -2433,7 +2475,7 @@
         <v>31</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="O27" s="1" t="s">
         <v>33</v>
@@ -2442,10 +2484,10 @@
         <v>34</v>
       </c>
       <c r="Q27" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R27" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
@@ -2453,31 +2495,31 @@
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>123</v>
+        <v>155</v>
       </c>
       <c r="K28" s="1" t="s">
         <v>29</v>
@@ -2486,10 +2528,10 @@
         <v>30</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="O28" s="1" t="s">
         <v>33</v>
@@ -2498,10 +2540,10 @@
         <v>34</v>
       </c>
       <c r="Q28" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R28" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
@@ -2509,31 +2551,31 @@
         <v>19</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>152</v>
+        <v>44</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>154</v>
+        <v>124</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>155</v>
+        <v>69</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>156</v>
+        <v>70</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>157</v>
+        <v>125</v>
       </c>
       <c r="K29" s="1" t="s">
         <v>29</v>
@@ -2545,7 +2587,7 @@
         <v>31</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="O29" s="1" t="s">
         <v>33</v>
@@ -2554,10 +2596,10 @@
         <v>34</v>
       </c>
       <c r="Q29" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R29" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
@@ -2565,31 +2607,31 @@
         <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>115</v>
+        <v>35</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>118</v>
+        <v>39</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>119</v>
+        <v>40</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="K30" s="1" t="s">
         <v>29</v>
@@ -2598,10 +2640,10 @@
         <v>30</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="O30" s="1" t="s">
         <v>33</v>
@@ -2610,10 +2652,10 @@
         <v>34</v>
       </c>
       <c r="Q30" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R30" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
@@ -2621,31 +2663,31 @@
         <v>19</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>160</v>
+        <v>35</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F31" s="1" t="s">
-        <v>99</v>
-      </c>
       <c r="G31" s="1" t="s">
-        <v>100</v>
+        <v>39</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>101</v>
+        <v>40</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>96</v>
+        <v>28</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>29</v>
@@ -2654,10 +2696,10 @@
         <v>30</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>33</v>
@@ -2666,10 +2708,10 @@
         <v>34</v>
       </c>
       <c r="Q31" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R31" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
@@ -2677,31 +2719,31 @@
         <v>19</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="G32" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>87</v>
-      </c>
       <c r="H32" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="K32" s="1" t="s">
         <v>29</v>
@@ -2710,10 +2752,10 @@
         <v>30</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O32" s="1" t="s">
         <v>33</v>
@@ -2722,10 +2764,10 @@
         <v>34</v>
       </c>
       <c r="Q32" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R32" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
@@ -2733,31 +2775,31 @@
         <v>19</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>115</v>
+        <v>166</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>118</v>
+        <v>169</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>119</v>
+        <v>170</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="K33" s="1" t="s">
         <v>29</v>
@@ -2766,10 +2808,10 @@
         <v>30</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>33</v>
@@ -2778,10 +2820,10 @@
         <v>34</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R33" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
@@ -2789,31 +2831,31 @@
         <v>19</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>115</v>
+        <v>35</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>118</v>
+        <v>39</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>119</v>
+        <v>40</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="K34" s="1" t="s">
         <v>29</v>
@@ -2822,10 +2864,10 @@
         <v>30</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>50</v>
+        <v>102</v>
       </c>
       <c r="O34" s="1" t="s">
         <v>33</v>
@@ -2834,10 +2876,10 @@
         <v>34</v>
       </c>
       <c r="Q34" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R34" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
@@ -2845,31 +2887,31 @@
         <v>19</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>171</v>
+        <v>119</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>94</v>
+        <v>120</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>95</v>
+        <v>121</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>41</v>
+        <v>117</v>
       </c>
       <c r="K35" s="1" t="s">
         <v>29</v>
@@ -2878,10 +2920,10 @@
         <v>30</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>32</v>
+        <v>102</v>
       </c>
       <c r="O35" s="1" t="s">
         <v>33</v>
@@ -2890,10 +2932,10 @@
         <v>34</v>
       </c>
       <c r="Q35" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R35" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
@@ -2901,31 +2943,31 @@
         <v>19</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>173</v>
+        <v>99</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="K36" s="1" t="s">
         <v>29</v>
@@ -2934,10 +2976,10 @@
         <v>30</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="O36" s="1" t="s">
         <v>33</v>
@@ -2946,10 +2988,10 @@
         <v>34</v>
       </c>
       <c r="Q36" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
@@ -2957,31 +2999,31 @@
         <v>19</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="K37" s="1" t="s">
         <v>29</v>
@@ -2990,10 +3032,10 @@
         <v>30</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O37" s="1" t="s">
         <v>33</v>
@@ -3002,10 +3044,10 @@
         <v>34</v>
       </c>
       <c r="Q37" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R37" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
@@ -3013,31 +3055,31 @@
         <v>19</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>97</v>
+        <v>35</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="K38" s="1" t="s">
         <v>29</v>
@@ -3046,10 +3088,10 @@
         <v>30</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="O38" s="1" t="s">
         <v>33</v>
@@ -3058,10 +3100,10 @@
         <v>34</v>
       </c>
       <c r="Q38" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="R38" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
@@ -3069,55 +3111,279 @@
         <v>19</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>72</v>
+        <v>174</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>63</v>
+        <v>26</v>
       </c>
       <c r="I39" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>123</v>
+        <v>71</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>65</v>
+        <v>29</v>
       </c>
       <c r="L39" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M39" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N39" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="M39" s="1" t="s">
+      <c r="O39" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P39" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q39" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R39" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="N39" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="O39" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="P39" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q39" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="R39" s="1" t="s">
-        <v>35</v>
+      <c r="C40" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L40" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="N40" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O40" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P40" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q40" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R40" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L41" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="N41" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O41" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P41" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q41" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R41" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L42" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M42" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N42" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="O42" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P42" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q42" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R42" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M43" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N43" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P43" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q43" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R43" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update 實價登錄 data to 44 transactions (2026/09/03 query)
Replace data/guoyang_boyu_實價登錄.xlsx with the latest export (41 ->
44 records) and regenerate. New transactions: A9 12F (1,929萬), A13
12F (3,188萬), B2 18F (1,799萬). Move NEW_SINCE_DATE to 115/07/10 (the
previous snapshot's newest date) so just these three are highlighted
this round.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019qMmeph4mJXozC5k1Nyzof
</commit_message>
<xml_diff>
--- a/data/guoyang_boyu_實價登錄.xlsx
+++ b/data/guoyang_boyu_實價登錄.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="195">
-  <si>
-    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,114 年 8 月 至115 年 8 月 ,建案名稱：國揚鉑御　　　　　　資料來源：不動產交易實價查詢服務網　2026年08月22日 13:59:31</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="202">
+  <si>
+    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,114 年 8 月 至115 年 8 月 ,建案名稱：國揚鉑御　　　　　　資料來源：不動產交易實價查詢服務網　2026年09月04日 01:34:35</t>
   </si>
   <si>
     <t>建物坐落</t>
@@ -82,45 +82,102 @@
     <t>國揚鉑御</t>
   </si>
   <si>
+    <t>115/07/18　</t>
+  </si>
+  <si>
+    <t>1929</t>
+  </si>
+  <si>
+    <t>73.7</t>
+  </si>
+  <si>
+    <t>29.41</t>
+  </si>
+  <si>
+    <t>40.97%</t>
+  </si>
+  <si>
+    <t>住宅大樓(11層含以上有電梯)</t>
+  </si>
+  <si>
+    <t>　12/20　</t>
+  </si>
+  <si>
+    <t>房地(土地+建物)+車位</t>
+  </si>
+  <si>
+    <t>土:1 建:1車:1</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>280</t>
+  </si>
+  <si>
+    <t>住家用</t>
+  </si>
+  <si>
+    <t>鋼筋混凝土造</t>
+  </si>
+  <si>
+    <t>B棟2號</t>
+  </si>
+  <si>
+    <t>115/07/15　</t>
+  </si>
+  <si>
+    <t>1799</t>
+  </si>
+  <si>
+    <t>68.46</t>
+  </si>
+  <si>
+    <t>29.51</t>
+  </si>
+  <si>
+    <t>40.84%</t>
+  </si>
+  <si>
+    <t>　18/20　</t>
+  </si>
+  <si>
+    <t>260</t>
+  </si>
+  <si>
+    <t>A棟13號</t>
+  </si>
+  <si>
+    <t>115/07/14　</t>
+  </si>
+  <si>
+    <t>3188</t>
+  </si>
+  <si>
+    <t>71.68</t>
+  </si>
+  <si>
+    <t>48.02</t>
+  </si>
+  <si>
+    <t>46.98%</t>
+  </si>
+  <si>
+    <t>3房2廳2衛</t>
+  </si>
+  <si>
+    <t>250</t>
+  </si>
+  <si>
     <t>115/07/10　</t>
   </si>
   <si>
     <t>1854</t>
   </si>
   <si>
-    <t>71.68</t>
-  </si>
-  <si>
-    <t>29.41</t>
-  </si>
-  <si>
-    <t>40.97%</t>
-  </si>
-  <si>
-    <t>住宅大樓(11層含以上有電梯)</t>
-  </si>
-  <si>
     <t>　6/20　</t>
   </si>
   <si>
-    <t>房地(土地+建物)+車位</t>
-  </si>
-  <si>
-    <t>土:1 建:1車:1</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>250</t>
-  </si>
-  <si>
-    <t>住家用</t>
-  </si>
-  <si>
-    <t>鋼筋混凝土造</t>
-  </si>
-  <si>
     <t>B棟9號</t>
   </si>
   <si>
@@ -142,12 +199,12 @@
     <t>　3/20　</t>
   </si>
   <si>
-    <t>3房2廳2衛</t>
-  </si>
-  <si>
     <t>230</t>
   </si>
   <si>
+    <t>1150731全部解約</t>
+  </si>
+  <si>
     <t>A棟15號</t>
   </si>
   <si>
@@ -163,9 +220,6 @@
     <t>58.08%</t>
   </si>
   <si>
-    <t>　12/20　</t>
-  </si>
-  <si>
     <t>房地(土地+建物)</t>
   </si>
   <si>
@@ -190,9 +244,6 @@
     <t>47.58%</t>
   </si>
   <si>
-    <t>280</t>
-  </si>
-  <si>
     <t>B棟8號</t>
   </si>
   <si>
@@ -256,9 +307,6 @@
     <t>　10/20　</t>
   </si>
   <si>
-    <t>A棟13號</t>
-  </si>
-  <si>
     <t>115/06/20　</t>
   </si>
   <si>
@@ -268,18 +316,6 @@
     <t>74.39</t>
   </si>
   <si>
-    <t>48.02</t>
-  </si>
-  <si>
-    <t>46.98%</t>
-  </si>
-  <si>
-    <t>　18/20　</t>
-  </si>
-  <si>
-    <t>B棟2號</t>
-  </si>
-  <si>
     <t>115/06/19　</t>
   </si>
   <si>
@@ -308,21 +344,6 @@
   </si>
   <si>
     <t>115/06/06　</t>
-  </si>
-  <si>
-    <t>1799</t>
-  </si>
-  <si>
-    <t>68.46</t>
-  </si>
-  <si>
-    <t>29.51</t>
-  </si>
-  <si>
-    <t>40.84%</t>
-  </si>
-  <si>
-    <t>260</t>
   </si>
   <si>
     <t>115/06/03　</t>
@@ -990,26 +1011,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R43"/>
+  <dimension ref="A1:R46"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="50.63408000000001" customWidth="1"/>
-    <col min="2" max="2" width="15.389080000000002" customWidth="1"/>
-    <col min="3" max="3" width="16.50474" customWidth="1"/>
-    <col min="4" max="4" width="20.59316" customWidth="1"/>
-    <col min="5" max="5" width="19.177760000000003" customWidth="1"/>
-    <col min="6" max="6" width="16.27934" customWidth="1"/>
-    <col min="7" max="7" width="12.488434000000002" customWidth="1"/>
-    <col min="8" max="8" width="20.518680000000003" customWidth="1"/>
-    <col min="9" max="9" width="51.15026" customWidth="1"/>
-    <col min="10" max="10" width="17.620260000000002" customWidth="1"/>
-    <col min="11" max="11" width="39.76868" customWidth="1"/>
-    <col min="12" max="12" width="22.863680000000002" customWidth="1"/>
-    <col min="13" max="13" width="18.51066" customWidth="1"/>
-    <col min="14" max="15" width="16.50474" customWidth="1"/>
-    <col min="16" max="16" width="24.535000000000004" customWidth="1"/>
-    <col min="17" max="17" width="16.50474" customWidth="1"/>
-    <col min="18" max="18" width="8.491868" customWidth="1"/>
+    <col min="1" max="1" width="48.96934" customWidth="1"/>
+    <col min="2" max="2" width="14.872760000000001" customWidth="1"/>
+    <col min="3" max="3" width="15.94908" customWidth="1"/>
+    <col min="4" max="4" width="19.90632" customWidth="1"/>
+    <col min="5" max="5" width="18.53684" customWidth="1"/>
+    <col min="6" max="6" width="15.732500000000002" customWidth="1"/>
+    <col min="7" max="7" width="12.064066" customWidth="1"/>
+    <col min="8" max="8" width="19.83408" customWidth="1"/>
+    <col min="9" max="9" width="49.47026" customWidth="1"/>
+    <col min="10" max="10" width="17.029740000000004" customWidth="1"/>
+    <col min="11" max="11" width="38.45842" customWidth="1"/>
+    <col min="12" max="12" width="22.102500000000003" customWidth="1"/>
+    <col min="13" max="13" width="17.89158" customWidth="1"/>
+    <col min="14" max="15" width="15.94908" customWidth="1"/>
+    <col min="16" max="16" width="23.71908" customWidth="1"/>
+    <col min="17" max="17" width="29.402240000000003" customWidth="1"/>
+    <col min="18" max="18" width="8.203132000000002" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -1184,10 +1205,10 @@
         <v>30</v>
       </c>
       <c r="M4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N4" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="O4" s="1" t="s">
         <v>33</v>
@@ -1207,13 +1228,13 @@
         <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>45</v>
@@ -1231,19 +1252,19 @@
         <v>27</v>
       </c>
       <c r="J5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M5" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="N5" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>33</v>
@@ -1263,32 +1284,32 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="K6" s="1" t="s">
         <v>29</v>
       </c>
@@ -1296,10 +1317,10 @@
         <v>30</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>33</v>
@@ -1319,52 +1340,52 @@
         <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="1" t="s">
+      <c r="I7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="K7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N7" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="O7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q7" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="R7" s="1" t="s">
         <v>31</v>
@@ -1375,43 +1396,43 @@
         <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="I8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K8" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="L8" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="M8" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>33</v>
@@ -1431,31 +1452,31 @@
         <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="I9" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>29</v>
@@ -1464,10 +1485,10 @@
         <v>30</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>33</v>
@@ -1487,43 +1508,43 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="I10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="K10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N10" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="N10" s="1" t="s">
-        <v>66</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>33</v>
@@ -1543,43 +1564,43 @@
         <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="H11" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="1" t="s">
+      <c r="I11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="K11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N11" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>33</v>
@@ -1599,43 +1620,43 @@
         <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="I12" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>33</v>
@@ -1655,7 +1676,7 @@
         <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>21</v>
@@ -1670,16 +1691,16 @@
         <v>99</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>100</v>
+        <v>47</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>101</v>
+        <v>48</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>86</v>
+        <v>41</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>29</v>
@@ -1688,10 +1709,10 @@
         <v>30</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="O13" s="1" t="s">
         <v>33</v>
@@ -1711,43 +1732,43 @@
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>93</v>
+        <v>35</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H14" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="I14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J14" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G14" s="1" t="s">
+      <c r="K14" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L14" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="M14" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>33</v>
@@ -1767,43 +1788,43 @@
         <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>108</v>
-      </c>
       <c r="F15" s="1" t="s">
-        <v>109</v>
+        <v>85</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>111</v>
+        <v>67</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>33</v>
@@ -1823,31 +1844,31 @@
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>115</v>
+        <v>37</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>29</v>
@@ -1859,7 +1880,7 @@
         <v>31</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>102</v>
+        <v>42</v>
       </c>
       <c r="O16" s="1" t="s">
         <v>33</v>
@@ -1879,31 +1900,31 @@
         <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>120</v>
+        <v>86</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>121</v>
+        <v>87</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>29</v>
@@ -1915,7 +1936,7 @@
         <v>31</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="O17" s="1" t="s">
         <v>33</v>
@@ -1935,31 +1956,31 @@
         <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>69</v>
+        <v>117</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>70</v>
+        <v>118</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="K18" s="1" t="s">
         <v>29</v>
@@ -1968,10 +1989,10 @@
         <v>30</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="O18" s="1" t="s">
         <v>33</v>
@@ -1991,31 +2012,31 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>73</v>
+        <v>120</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>78</v>
+        <v>26</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>29</v>
@@ -2024,10 +2045,10 @@
         <v>30</v>
       </c>
       <c r="M19" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N19" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="N19" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="O19" s="1" t="s">
         <v>33</v>
@@ -2047,31 +2068,31 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>29</v>
@@ -2080,10 +2101,10 @@
         <v>30</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>33</v>
@@ -2103,7 +2124,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>21</v>
@@ -2112,22 +2133,22 @@
         <v>129</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>39</v>
+        <v>86</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>40</v>
+        <v>87</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>79</v>
+        <v>132</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>29</v>
@@ -2136,10 +2157,10 @@
         <v>30</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>33</v>
@@ -2159,31 +2180,31 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>29</v>
@@ -2192,10 +2213,10 @@
         <v>30</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="O22" s="1" t="s">
         <v>33</v>
@@ -2215,32 +2236,32 @@
         <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="H23" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="I23" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J23" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="K23" s="1" t="s">
         <v>29</v>
       </c>
@@ -2248,7 +2269,7 @@
         <v>30</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="N23" s="1" t="s">
         <v>32</v>
@@ -2271,31 +2292,31 @@
         <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>144</v>
-      </c>
       <c r="G24" s="1" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>145</v>
+        <v>96</v>
       </c>
       <c r="K24" s="1" t="s">
         <v>29</v>
@@ -2304,10 +2325,10 @@
         <v>30</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="O24" s="1" t="s">
         <v>33</v>
@@ -2327,43 +2348,43 @@
         <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>148</v>
-      </c>
       <c r="G25" s="1" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J25" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M25" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K25" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="N25" s="1" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="O25" s="1" t="s">
         <v>33</v>
@@ -2383,43 +2404,43 @@
         <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>150</v>
-      </c>
       <c r="G26" s="1" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="K26" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N26" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="L26" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="M26" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N26" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="O26" s="1" t="s">
         <v>33</v>
@@ -2439,32 +2460,32 @@
         <v>19</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J27" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="K27" s="1" t="s">
         <v>29</v>
       </c>
@@ -2472,10 +2493,10 @@
         <v>30</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="O27" s="1" t="s">
         <v>33</v>
@@ -2495,31 +2516,31 @@
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>155</v>
+        <v>28</v>
       </c>
       <c r="K28" s="1" t="s">
         <v>29</v>
@@ -2528,10 +2549,10 @@
         <v>30</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="O28" s="1" t="s">
         <v>33</v>
@@ -2551,43 +2572,43 @@
         <v>19</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="F29" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="G29" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L29" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="H29" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L29" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="M29" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O29" s="1" t="s">
         <v>33</v>
@@ -2607,31 +2628,31 @@
         <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="F30" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="F30" s="1" t="s">
-        <v>160</v>
-      </c>
       <c r="G30" s="1" t="s">
-        <v>39</v>
+        <v>86</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>40</v>
+        <v>87</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="K30" s="1" t="s">
         <v>29</v>
@@ -2640,10 +2661,10 @@
         <v>30</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="O30" s="1" t="s">
         <v>33</v>
@@ -2663,32 +2684,32 @@
         <v>19</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="E31" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J31" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="G31" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H31" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="K31" s="1" t="s">
         <v>29</v>
       </c>
@@ -2696,10 +2717,10 @@
         <v>30</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>33</v>
@@ -2719,7 +2740,7 @@
         <v>19</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>21</v>
@@ -2731,19 +2752,19 @@
         <v>164</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>165</v>
+        <v>131</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>28</v>
+        <v>132</v>
       </c>
       <c r="K32" s="1" t="s">
         <v>29</v>
@@ -2752,10 +2773,10 @@
         <v>30</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="O32" s="1" t="s">
         <v>33</v>
@@ -2775,31 +2796,31 @@
         <v>19</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="E33" s="1" t="s">
+      <c r="F33" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="F33" s="1" t="s">
-        <v>168</v>
-      </c>
       <c r="G33" s="1" t="s">
-        <v>169</v>
+        <v>58</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>170</v>
+        <v>59</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>171</v>
+        <v>88</v>
       </c>
       <c r="K33" s="1" t="s">
         <v>29</v>
@@ -2808,10 +2829,10 @@
         <v>30</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>33</v>
@@ -2831,31 +2852,31 @@
         <v>19</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="K34" s="1" t="s">
         <v>29</v>
@@ -2864,10 +2885,10 @@
         <v>30</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>102</v>
+        <v>50</v>
       </c>
       <c r="O34" s="1" t="s">
         <v>33</v>
@@ -2887,31 +2908,31 @@
         <v>19</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>174</v>
+        <v>43</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>119</v>
+        <v>172</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>120</v>
+        <v>47</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>121</v>
+        <v>48</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>117</v>
+        <v>53</v>
       </c>
       <c r="K35" s="1" t="s">
         <v>29</v>
@@ -2920,10 +2941,10 @@
         <v>30</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>102</v>
+        <v>32</v>
       </c>
       <c r="O35" s="1" t="s">
         <v>33</v>
@@ -2943,31 +2964,31 @@
         <v>19</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>107</v>
+        <v>173</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D36" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="F36" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="G36" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="H36" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F36" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>111</v>
-      </c>
       <c r="I36" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>86</v>
+        <v>178</v>
       </c>
       <c r="K36" s="1" t="s">
         <v>29</v>
@@ -2976,10 +2997,10 @@
         <v>30</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="O36" s="1" t="s">
         <v>33</v>
@@ -2999,31 +3020,31 @@
         <v>19</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>180</v>
+        <v>82</v>
       </c>
       <c r="K37" s="1" t="s">
         <v>29</v>
@@ -3032,10 +3053,10 @@
         <v>30</v>
       </c>
       <c r="M37" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N37" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="N37" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="O37" s="1" t="s">
         <v>33</v>
@@ -3055,31 +3076,31 @@
         <v>19</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>35</v>
+        <v>181</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>182</v>
+        <v>126</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>39</v>
+        <v>127</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>40</v>
+        <v>128</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="K38" s="1" t="s">
         <v>29</v>
@@ -3088,10 +3109,10 @@
         <v>30</v>
       </c>
       <c r="M38" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N38" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="N38" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="O38" s="1" t="s">
         <v>33</v>
@@ -3111,31 +3132,31 @@
         <v>19</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>174</v>
+        <v>114</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>184</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>185</v>
+        <v>38</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>25</v>
+        <v>117</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>26</v>
+        <v>118</v>
       </c>
       <c r="I39" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="K39" s="1" t="s">
         <v>29</v>
@@ -3144,10 +3165,10 @@
         <v>30</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="O39" s="1" t="s">
         <v>33</v>
@@ -3167,32 +3188,32 @@
         <v>19</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E40" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J40" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G40" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I40" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="K40" s="1" t="s">
         <v>29</v>
       </c>
@@ -3200,7 +3221,7 @@
         <v>30</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="N40" s="1" t="s">
         <v>32</v>
@@ -3223,31 +3244,31 @@
         <v>19</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="F41" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="F41" s="1" t="s">
-        <v>190</v>
-      </c>
       <c r="G41" s="1" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>145</v>
+        <v>41</v>
       </c>
       <c r="K41" s="1" t="s">
         <v>29</v>
@@ -3256,10 +3277,10 @@
         <v>30</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="O41" s="1" t="s">
         <v>33</v>
@@ -3279,13 +3300,13 @@
         <v>19</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>20</v>
+        <v>181</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>191</v>
@@ -3303,7 +3324,7 @@
         <v>27</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="K42" s="1" t="s">
         <v>29</v>
@@ -3315,7 +3336,7 @@
         <v>31</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="O42" s="1" t="s">
         <v>33</v>
@@ -3335,13 +3356,13 @@
         <v>19</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>96</v>
+        <v>54</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>193</v>
@@ -3350,39 +3371,207 @@
         <v>194</v>
       </c>
       <c r="G43" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M43" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N43" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P43" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q43" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R43" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="H43" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="I43" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K43" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L43" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="M43" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N43" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="O43" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="P43" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q43" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="R43" s="1" t="s">
+      <c r="C44" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K44" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L44" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M44" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N44" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O44" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P44" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q44" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R44" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J45" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="K45" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L45" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M45" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N45" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="O45" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P45" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q45" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R45" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="M46" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N46" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P46" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q46" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R46" s="1" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 實價登錄 data to 48 transactions (2026/09/16 query)
Replace data/guoyang_boyu_實價登錄.xlsx with the latest export (44 ->
48 records) and regenerate. New transactions: A8 14F (3,429萬), A9
14F (1,937萬), B5 18F (1,528萬) — B5's first-ever sale, B7 17F
(2,825萬). Move NEW_SINCE_DATE to 115/07/18 (the previous snapshot's
newest date) so just these four are highlighted this round.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019qMmeph4mJXozC5k1Nyzof
</commit_message>
<xml_diff>
--- a/data/guoyang_boyu_實價登錄.xlsx
+++ b/data/guoyang_boyu_實價登錄.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="202">
-  <si>
-    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,114 年 8 月 至115 年 8 月 ,建案名稱：國揚鉑御　　　　　　資料來源：不動產交易實價查詢服務網　2026年09月04日 01:34:35</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="213">
+  <si>
+    <t>預售屋案件:高雄市鼓山區房地(土地+建物),房地(土地+建物)+車位,114 年 8 月 至115 年 8 月 ,建案名稱：國揚鉑御　　　　　　資料來源：不動產交易實價查詢服務網　2026年09月16日 08:30:05</t>
   </si>
   <si>
     <t>建物坐落</t>
@@ -76,10 +76,118 @@
     <t>鼓山區龍中段194地號</t>
   </si>
   <si>
+    <t>A棟8號</t>
+  </si>
+  <si>
+    <t>國揚鉑御</t>
+  </si>
+  <si>
+    <t>115/07/29　</t>
+  </si>
+  <si>
+    <t>3429</t>
+  </si>
+  <si>
+    <t>70.97</t>
+  </si>
+  <si>
+    <t>51.41</t>
+  </si>
+  <si>
+    <t>47.74%</t>
+  </si>
+  <si>
+    <t>住宅大樓(11層含以上有電梯)</t>
+  </si>
+  <si>
+    <t>　14/20　</t>
+  </si>
+  <si>
+    <t>房地(土地+建物)+車位</t>
+  </si>
+  <si>
+    <t>土:1 建:1車:1</t>
+  </si>
+  <si>
+    <t>3房2廳2衛</t>
+  </si>
+  <si>
+    <t>280</t>
+  </si>
+  <si>
+    <t>住家用</t>
+  </si>
+  <si>
+    <t>鋼筋混凝土造</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>A棟9號</t>
   </si>
   <si>
-    <t>國揚鉑御</t>
+    <t>1937</t>
+  </si>
+  <si>
+    <t>74.5</t>
+  </si>
+  <si>
+    <t>29.41</t>
+  </si>
+  <si>
+    <t>40.97%</t>
+  </si>
+  <si>
+    <t>270</t>
+  </si>
+  <si>
+    <t>B棟5號</t>
+  </si>
+  <si>
+    <t>115/07/28　</t>
+  </si>
+  <si>
+    <t>1528</t>
+  </si>
+  <si>
+    <t>67.97</t>
+  </si>
+  <si>
+    <t>22.48</t>
+  </si>
+  <si>
+    <t>53.62%</t>
+  </si>
+  <si>
+    <t>　18/20　</t>
+  </si>
+  <si>
+    <t>房地(土地+建物)</t>
+  </si>
+  <si>
+    <t>土:1 建:1車:0</t>
+  </si>
+  <si>
+    <t>B棟7號</t>
+  </si>
+  <si>
+    <t>115/07/26　</t>
+  </si>
+  <si>
+    <t>2825</t>
+  </si>
+  <si>
+    <t>66.28</t>
+  </si>
+  <si>
+    <t>45.43</t>
+  </si>
+  <si>
+    <t>46.20%</t>
+  </si>
+  <si>
+    <t>　17/20　</t>
   </si>
   <si>
     <t>115/07/18　</t>
@@ -91,36 +199,9 @@
     <t>73.7</t>
   </si>
   <si>
-    <t>29.41</t>
-  </si>
-  <si>
-    <t>40.97%</t>
-  </si>
-  <si>
-    <t>住宅大樓(11層含以上有電梯)</t>
-  </si>
-  <si>
     <t>　12/20　</t>
   </si>
   <si>
-    <t>房地(土地+建物)+車位</t>
-  </si>
-  <si>
-    <t>土:1 建:1車:1</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>280</t>
-  </si>
-  <si>
-    <t>住家用</t>
-  </si>
-  <si>
-    <t>鋼筋混凝土造</t>
-  </si>
-  <si>
     <t>B棟2號</t>
   </si>
   <si>
@@ -139,9 +220,6 @@
     <t>40.84%</t>
   </si>
   <si>
-    <t>　18/20　</t>
-  </si>
-  <si>
     <t>260</t>
   </si>
   <si>
@@ -163,9 +241,6 @@
     <t>46.98%</t>
   </si>
   <si>
-    <t>3房2廳2衛</t>
-  </si>
-  <si>
     <t>250</t>
   </si>
   <si>
@@ -220,12 +295,6 @@
     <t>58.08%</t>
   </si>
   <si>
-    <t>房地(土地+建物)</t>
-  </si>
-  <si>
-    <t>土:1 建:1車:0</t>
-  </si>
-  <si>
     <t>A棟7號</t>
   </si>
   <si>
@@ -265,9 +334,6 @@
     <t>　16/20　</t>
   </si>
   <si>
-    <t>270</t>
-  </si>
-  <si>
     <t>1546</t>
   </si>
   <si>
@@ -286,9 +352,6 @@
     <t>240</t>
   </si>
   <si>
-    <t>A棟8號</t>
-  </si>
-  <si>
     <t>115/06/23　</t>
   </si>
   <si>
@@ -298,12 +361,6 @@
     <t>69.37</t>
   </si>
   <si>
-    <t>51.41</t>
-  </si>
-  <si>
-    <t>47.74%</t>
-  </si>
-  <si>
     <t>　10/20　</t>
   </si>
   <si>
@@ -322,12 +379,6 @@
     <t>1380</t>
   </si>
   <si>
-    <t>22.48</t>
-  </si>
-  <si>
-    <t>53.62%</t>
-  </si>
-  <si>
     <t>　2/20　</t>
   </si>
   <si>
@@ -535,21 +586,6 @@
     <t>69.68</t>
   </si>
   <si>
-    <t>B棟7號</t>
-  </si>
-  <si>
-    <t>2825</t>
-  </si>
-  <si>
-    <t>66.28</t>
-  </si>
-  <si>
-    <t>45.43</t>
-  </si>
-  <si>
-    <t>46.20%</t>
-  </si>
-  <si>
     <t>　19/20　</t>
   </si>
   <si>
@@ -575,9 +611,6 @@
   </si>
   <si>
     <t>66.78</t>
-  </si>
-  <si>
-    <t>　17/20　</t>
   </si>
   <si>
     <t>2806</t>
@@ -1011,7 +1044,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R46"/>
+  <dimension ref="A1:R50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="48.96934" customWidth="1"/>
@@ -1161,10 +1194,10 @@
         <v>34</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -1172,13 +1205,13 @@
         <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>37</v>
@@ -1196,20 +1229,20 @@
         <v>27</v>
       </c>
       <c r="J4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="O4" s="1" t="s">
         <v>33</v>
       </c>
@@ -1217,10 +1250,10 @@
         <v>34</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -1228,43 +1261,43 @@
         <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="K5" s="1" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>33</v>
@@ -1273,10 +1306,10 @@
         <v>34</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -1284,31 +1317,31 @@
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>29</v>
@@ -1320,7 +1353,7 @@
         <v>31</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>33</v>
@@ -1329,10 +1362,10 @@
         <v>34</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
@@ -1340,31 +1373,31 @@
         <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>29</v>
@@ -1373,10 +1406,10 @@
         <v>30</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>33</v>
@@ -1385,10 +1418,10 @@
         <v>34</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>62</v>
+        <v>35</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
@@ -1396,13 +1429,13 @@
         <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>64</v>
@@ -1420,20 +1453,20 @@
         <v>27</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="K8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N8" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="L8" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="O8" s="1" t="s">
         <v>33</v>
       </c>
@@ -1441,10 +1474,10 @@
         <v>34</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
@@ -1452,44 +1485,44 @@
         <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N9" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="I9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="O9" s="1" t="s">
         <v>33</v>
       </c>
@@ -1497,10 +1530,10 @@
         <v>34</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -1508,32 +1541,32 @@
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="K10" s="1" t="s">
         <v>29</v>
       </c>
@@ -1541,10 +1574,10 @@
         <v>30</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>33</v>
@@ -1553,10 +1586,10 @@
         <v>34</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
@@ -1564,31 +1597,31 @@
         <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H11" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="I11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>29</v>
@@ -1600,7 +1633,7 @@
         <v>31</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>33</v>
@@ -1609,10 +1642,10 @@
         <v>34</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
@@ -1620,43 +1653,43 @@
         <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I12" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>33</v>
@@ -1665,10 +1698,10 @@
         <v>34</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
@@ -1676,31 +1709,31 @@
         <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="I13" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>29</v>
@@ -1709,10 +1742,10 @@
         <v>30</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="O13" s="1" t="s">
         <v>33</v>
@@ -1721,10 +1754,10 @@
         <v>34</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -1732,7 +1765,7 @@
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>21</v>
@@ -1744,31 +1777,31 @@
         <v>101</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="M14" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>33</v>
@@ -1777,10 +1810,10 @@
         <v>34</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
@@ -1788,43 +1821,43 @@
         <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="G15" s="1" t="s">
-        <v>66</v>
+        <v>108</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>67</v>
+        <v>109</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>88</v>
+        <v>110</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>31</v>
+        <v>111</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>33</v>
@@ -1833,10 +1866,10 @@
         <v>34</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
@@ -1844,31 +1877,31 @@
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>108</v>
+        <v>20</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>38</v>
+        <v>114</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>41</v>
+        <v>115</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>29</v>
@@ -1880,7 +1913,7 @@
         <v>31</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="O16" s="1" t="s">
         <v>33</v>
@@ -1889,10 +1922,10 @@
         <v>34</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
@@ -1900,31 +1933,31 @@
         <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>113</v>
+        <v>48</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>29</v>
@@ -1936,7 +1969,7 @@
         <v>31</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="O17" s="1" t="s">
         <v>33</v>
@@ -1945,10 +1978,10 @@
         <v>34</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
@@ -1956,43 +1989,43 @@
         <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>114</v>
+        <v>62</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>117</v>
+        <v>46</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>118</v>
+        <v>47</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="O18" s="1" t="s">
         <v>33</v>
@@ -2001,10 +2034,10 @@
         <v>34</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
@@ -2012,43 +2045,43 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="O19" s="1" t="s">
         <v>33</v>
@@ -2057,10 +2090,10 @@
         <v>34</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
@@ -2068,31 +2101,31 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>20</v>
+        <v>125</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>125</v>
+        <v>64</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>126</v>
+        <v>65</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>127</v>
+        <v>66</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>128</v>
+        <v>67</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>29</v>
@@ -2101,10 +2134,10 @@
         <v>30</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>33</v>
@@ -2113,10 +2146,10 @@
         <v>34</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
@@ -2124,32 +2157,32 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="G21" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J21" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>132</v>
-      </c>
       <c r="K21" s="1" t="s">
         <v>29</v>
       </c>
@@ -2157,10 +2190,10 @@
         <v>30</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>33</v>
@@ -2169,10 +2202,10 @@
         <v>34</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R21" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
@@ -2180,31 +2213,31 @@
         <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>90</v>
+        <v>131</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="H22" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="I22" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>41</v>
+        <v>136</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>29</v>
@@ -2213,7 +2246,7 @@
         <v>30</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N22" s="1" t="s">
         <v>32</v>
@@ -2225,10 +2258,10 @@
         <v>34</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
@@ -2236,25 +2269,25 @@
         <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>43</v>
+        <v>137</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>139</v>
+        <v>39</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>140</v>
+        <v>40</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>27</v>
@@ -2269,10 +2302,10 @@
         <v>30</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="O23" s="1" t="s">
         <v>33</v>
@@ -2281,10 +2314,10 @@
         <v>34</v>
       </c>
       <c r="Q23" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R23" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
@@ -2292,13 +2325,13 @@
         <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>142</v>
@@ -2307,16 +2340,16 @@
         <v>143</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>58</v>
+        <v>144</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>59</v>
+        <v>145</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>96</v>
+        <v>141</v>
       </c>
       <c r="K24" s="1" t="s">
         <v>29</v>
@@ -2325,10 +2358,10 @@
         <v>30</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="O24" s="1" t="s">
         <v>33</v>
@@ -2337,10 +2370,10 @@
         <v>34</v>
       </c>
       <c r="Q24" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R24" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
@@ -2348,31 +2381,31 @@
         <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>53</v>
+        <v>149</v>
       </c>
       <c r="K25" s="1" t="s">
         <v>29</v>
@@ -2381,10 +2414,10 @@
         <v>30</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="O25" s="1" t="s">
         <v>33</v>
@@ -2393,10 +2426,10 @@
         <v>34</v>
       </c>
       <c r="Q25" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
@@ -2404,19 +2437,19 @@
         <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>25</v>
@@ -2428,7 +2461,7 @@
         <v>27</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="K26" s="1" t="s">
         <v>29</v>
@@ -2440,7 +2473,7 @@
         <v>31</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="O26" s="1" t="s">
         <v>33</v>
@@ -2449,10 +2482,10 @@
         <v>34</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
@@ -2460,31 +2493,31 @@
         <v>19</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>43</v>
+        <v>69</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>47</v>
+        <v>156</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>48</v>
+        <v>157</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="K27" s="1" t="s">
         <v>29</v>
@@ -2493,7 +2526,7 @@
         <v>30</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N27" s="1" t="s">
         <v>32</v>
@@ -2505,10 +2538,10 @@
         <v>34</v>
       </c>
       <c r="Q27" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R27" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
@@ -2516,7 +2549,7 @@
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>21</v>
@@ -2525,22 +2558,22 @@
         <v>153</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>28</v>
+        <v>115</v>
       </c>
       <c r="K28" s="1" t="s">
         <v>29</v>
@@ -2549,7 +2582,7 @@
         <v>30</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N28" s="1" t="s">
         <v>32</v>
@@ -2561,10 +2594,10 @@
         <v>34</v>
       </c>
       <c r="Q28" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R28" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
@@ -2572,43 +2605,43 @@
         <v>19</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>105</v>
+        <v>20</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="M29" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="O29" s="1" t="s">
         <v>33</v>
@@ -2617,10 +2650,10 @@
         <v>34</v>
       </c>
       <c r="Q29" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R29" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
@@ -2628,31 +2661,31 @@
         <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>105</v>
+        <v>137</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>86</v>
+        <v>39</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="K30" s="1" t="s">
         <v>29</v>
@@ -2661,10 +2694,10 @@
         <v>30</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="O30" s="1" t="s">
         <v>33</v>
@@ -2673,10 +2706,10 @@
         <v>34</v>
       </c>
       <c r="Q30" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R30" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
@@ -2684,31 +2717,31 @@
         <v>19</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>29</v>
@@ -2717,10 +2750,10 @@
         <v>30</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>33</v>
@@ -2729,10 +2762,10 @@
         <v>34</v>
       </c>
       <c r="Q31" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R31" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
@@ -2740,31 +2773,31 @@
         <v>19</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>86</v>
+        <v>25</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>87</v>
+        <v>26</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>132</v>
+        <v>61</v>
       </c>
       <c r="K32" s="1" t="s">
         <v>29</v>
@@ -2776,7 +2809,7 @@
         <v>31</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="O32" s="1" t="s">
         <v>33</v>
@@ -2785,10 +2818,10 @@
         <v>34</v>
       </c>
       <c r="Q32" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R32" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
@@ -2796,43 +2829,43 @@
         <v>19</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>54</v>
+        <v>122</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>58</v>
+        <v>91</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>88</v>
+        <v>115</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>33</v>
@@ -2841,10 +2874,10 @@
         <v>34</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R33" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
@@ -2852,31 +2885,31 @@
         <v>19</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>54</v>
+        <v>122</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>58</v>
+        <v>108</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>59</v>
+        <v>109</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="K34" s="1" t="s">
         <v>29</v>
@@ -2885,10 +2918,10 @@
         <v>30</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="O34" s="1" t="s">
         <v>33</v>
@@ -2897,10 +2930,10 @@
         <v>34</v>
       </c>
       <c r="Q34" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R34" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
@@ -2908,7 +2941,7 @@
         <v>19</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>43</v>
+        <v>79</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>21</v>
@@ -2917,22 +2950,22 @@
         <v>170</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>53</v>
+        <v>179</v>
       </c>
       <c r="K35" s="1" t="s">
         <v>29</v>
@@ -2941,10 +2974,10 @@
         <v>30</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="O35" s="1" t="s">
         <v>33</v>
@@ -2953,10 +2986,10 @@
         <v>34</v>
       </c>
       <c r="Q35" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R35" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
@@ -2964,31 +2997,31 @@
         <v>19</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>173</v>
+        <v>88</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>175</v>
+        <v>148</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>176</v>
+        <v>108</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>177</v>
+        <v>109</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>178</v>
+        <v>149</v>
       </c>
       <c r="K36" s="1" t="s">
         <v>29</v>
@@ -2997,10 +3030,10 @@
         <v>30</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="O36" s="1" t="s">
         <v>33</v>
@@ -3009,10 +3042,10 @@
         <v>34</v>
       </c>
       <c r="Q36" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
@@ -3020,31 +3053,31 @@
         <v>19</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="K37" s="1" t="s">
         <v>29</v>
@@ -3053,10 +3086,10 @@
         <v>30</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="O37" s="1" t="s">
         <v>33</v>
@@ -3065,10 +3098,10 @@
         <v>34</v>
       </c>
       <c r="Q37" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R37" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
@@ -3076,7 +3109,7 @@
         <v>19</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>181</v>
+        <v>79</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>21</v>
@@ -3085,22 +3118,22 @@
         <v>182</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>126</v>
+        <v>186</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>127</v>
+        <v>83</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>128</v>
+        <v>84</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>124</v>
+        <v>78</v>
       </c>
       <c r="K38" s="1" t="s">
         <v>29</v>
@@ -3112,7 +3145,7 @@
         <v>31</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="O38" s="1" t="s">
         <v>33</v>
@@ -3121,10 +3154,10 @@
         <v>34</v>
       </c>
       <c r="Q38" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R38" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
@@ -3132,31 +3165,31 @@
         <v>19</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>114</v>
+        <v>69</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>38</v>
+        <v>189</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>117</v>
+        <v>73</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="I39" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="K39" s="1" t="s">
         <v>29</v>
@@ -3165,7 +3198,7 @@
         <v>30</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N39" s="1" t="s">
         <v>32</v>
@@ -3177,10 +3210,10 @@
         <v>34</v>
       </c>
       <c r="Q39" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R39" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
@@ -3188,31 +3221,31 @@
         <v>19</v>
       </c>
       <c r="B40" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>186</v>
-      </c>
       <c r="G40" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="I40" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="K40" s="1" t="s">
         <v>29</v>
@@ -3221,7 +3254,7 @@
         <v>30</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N40" s="1" t="s">
         <v>32</v>
@@ -3233,10 +3266,10 @@
         <v>34</v>
       </c>
       <c r="Q40" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R40" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
@@ -3244,31 +3277,31 @@
         <v>19</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>41</v>
+        <v>105</v>
       </c>
       <c r="K41" s="1" t="s">
         <v>29</v>
@@ -3277,10 +3310,10 @@
         <v>30</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="O41" s="1" t="s">
         <v>33</v>
@@ -3289,10 +3322,10 @@
         <v>34</v>
       </c>
       <c r="Q41" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R41" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
@@ -3300,31 +3333,31 @@
         <v>19</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>192</v>
+        <v>143</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>25</v>
+        <v>144</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>26</v>
+        <v>145</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>88</v>
+        <v>141</v>
       </c>
       <c r="K42" s="1" t="s">
         <v>29</v>
@@ -3333,10 +3366,10 @@
         <v>30</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="O42" s="1" t="s">
         <v>33</v>
@@ -3345,10 +3378,10 @@
         <v>34</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R42" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
@@ -3356,31 +3389,31 @@
         <v>19</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>54</v>
+        <v>131</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>194</v>
+        <v>65</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>58</v>
+        <v>134</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>59</v>
+        <v>135</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>152</v>
+        <v>48</v>
       </c>
       <c r="K43" s="1" t="s">
         <v>29</v>
@@ -3389,10 +3422,10 @@
         <v>30</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="O43" s="1" t="s">
         <v>33</v>
@@ -3401,10 +3434,10 @@
         <v>34</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R43" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
@@ -3412,31 +3445,31 @@
         <v>19</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>152</v>
+        <v>57</v>
       </c>
       <c r="K44" s="1" t="s">
         <v>29</v>
@@ -3445,7 +3478,7 @@
         <v>30</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="N44" s="1" t="s">
         <v>32</v>
@@ -3457,10 +3490,10 @@
         <v>34</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R44" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
@@ -3468,31 +3501,31 @@
         <v>19</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>26</v>
+        <v>84</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>27</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="K45" s="1" t="s">
         <v>29</v>
@@ -3504,7 +3537,7 @@
         <v>31</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="O45" s="1" t="s">
         <v>33</v>
@@ -3513,10 +3546,10 @@
         <v>34</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R45" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
@@ -3524,55 +3557,279 @@
         <v>19</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>108</v>
+        <v>193</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>21</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F46" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M46" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N46" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P46" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q46" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R46" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D47" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="G46" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="H46" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J46" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="K46" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="L46" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="M46" s="1" t="s">
+      <c r="E47" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L47" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M47" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N46" s="1" t="s">
+      <c r="N47" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="O47" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P47" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q47" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R47" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="K48" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L48" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M48" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="O46" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="P46" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q46" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="R46" s="1" t="s">
-        <v>31</v>
+      <c r="N48" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O48" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P48" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q48" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R48" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J49" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="K49" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L49" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M49" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N49" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O49" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P49" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q49" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R49" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="K50" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L50" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M50" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N50" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O50" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P50" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q50" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R50" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>